<commit_message>
V.3 Normalización de la base de datos
</commit_message>
<xml_diff>
--- a/Documentación/Trimestre III/Normalización Proyecto CheerClick.xlsx
+++ b/Documentación/Trimestre III/Normalización Proyecto CheerClick.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="256">
   <si>
     <t>Gestión de Usuarios</t>
   </si>
@@ -116,7 +116,7 @@
     <t>Id_usuario PK</t>
   </si>
   <si>
-    <t>Id_tipo PK</t>
+    <t>Id_tipoDoc PK</t>
   </si>
   <si>
     <t>Id_genero PK</t>
@@ -140,7 +140,7 @@
     <t>Id_PQRS              PK</t>
   </si>
   <si>
-    <t>Id_tipos                PK</t>
+    <t>Id_tiposPQRS     PK</t>
   </si>
   <si>
     <t>Id_respuesta            PK</t>
@@ -191,7 +191,7 @@
     <t>Id_condicion    PK</t>
   </si>
   <si>
-    <t>Id_tipo FK</t>
+    <t>Id_tipoDoc FK</t>
   </si>
   <si>
     <t>tipo_cc</t>
@@ -233,7 +233,7 @@
     <t>Id_usuario                         FK</t>
   </si>
   <si>
-    <t>Id_niveles                 FK</t>
+    <t>Id_tipo_horario  FK</t>
   </si>
   <si>
     <t>Id_horarios                      FK</t>
@@ -293,7 +293,7 @@
     <t>estaPago_vencido</t>
   </si>
   <si>
-    <t>Id_tipos               FK</t>
+    <t>Id_tiposPQRS       FK</t>
   </si>
   <si>
     <t>tipo_reclamo</t>
@@ -311,355 +311,346 @@
     <t>nive_atletas</t>
   </si>
   <si>
+    <t>Id_niveles        FK</t>
+  </si>
+  <si>
+    <t>dia_nombre</t>
+  </si>
+  <si>
+    <t>franja_inicio</t>
+  </si>
+  <si>
+    <t>Tip_competencia</t>
+  </si>
+  <si>
+    <t>ren_observaciones</t>
+  </si>
+  <si>
+    <t>asi_fechaAsis</t>
+  </si>
+  <si>
+    <t>Id_asistencia    FK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id_usuario    FK         </t>
+  </si>
+  <si>
+    <t>esta_noDisponible</t>
+  </si>
+  <si>
+    <t>Id_categoria    FK</t>
+  </si>
+  <si>
+    <t>cond_listoEntrega</t>
+  </si>
+  <si>
+    <t>Id_nivel FK</t>
+  </si>
+  <si>
+    <t>tipo_ti</t>
+  </si>
+  <si>
+    <t>gene_otro</t>
+  </si>
+  <si>
+    <t>rol_atleta</t>
+  </si>
+  <si>
+    <t>acu_apellido</t>
+  </si>
+  <si>
+    <t>Id_estadoPago     FK</t>
+  </si>
+  <si>
+    <t>estaPago_pendiente</t>
+  </si>
+  <si>
+    <t>PQRS_descripcion</t>
+  </si>
+  <si>
+    <t>tipo_sugerencia</t>
+  </si>
+  <si>
+    <t>res_respuesta</t>
+  </si>
+  <si>
+    <t>est_tramite</t>
+  </si>
+  <si>
+    <t>Prio_baja</t>
+  </si>
+  <si>
+    <t>nive_nombre</t>
+  </si>
+  <si>
     <t>hor_enfoque</t>
   </si>
   <si>
-    <t>dia_nombre</t>
-  </si>
-  <si>
-    <t>franja_inicio</t>
-  </si>
-  <si>
-    <t>Tip_competencia</t>
-  </si>
-  <si>
-    <t>ren_observaciones</t>
-  </si>
-  <si>
-    <t>asi_fechaAsis</t>
-  </si>
-  <si>
-    <t>Id_asistencia    FK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Id_usuario    FK         </t>
-  </si>
-  <si>
-    <t>esta_noDisponible</t>
+    <t>franja_fin</t>
+  </si>
+  <si>
+    <t>Tip_Refuerzo</t>
+  </si>
+  <si>
+    <t>ren_descripcionHabilidad</t>
+  </si>
+  <si>
+    <t>asi_justificacion</t>
+  </si>
+  <si>
+    <t>nove_presente</t>
+  </si>
+  <si>
+    <t>imple_nombre</t>
+  </si>
+  <si>
+    <t>Id_implemento   FK</t>
+  </si>
+  <si>
+    <t>cond_entregado</t>
+  </si>
+  <si>
+    <t>Id_rol  FK</t>
+  </si>
+  <si>
+    <t>tipo_pasa</t>
+  </si>
+  <si>
+    <t>acu_telefono</t>
+  </si>
+  <si>
+    <t>men_fechaPago</t>
+  </si>
+  <si>
+    <t>PQRS_fechaCrea</t>
+  </si>
+  <si>
+    <t>tipo_solicitud</t>
+  </si>
+  <si>
+    <t>res_fecha</t>
+  </si>
+  <si>
+    <t>Id_PQRS        FK</t>
+  </si>
+  <si>
+    <t>nive_entrenador</t>
+  </si>
+  <si>
+    <t>hor_indicaciones</t>
+  </si>
+  <si>
+    <t>Tip_fisico</t>
+  </si>
+  <si>
+    <t>ren_fecha</t>
+  </si>
+  <si>
+    <t>nove_falta</t>
+  </si>
+  <si>
+    <t>imple_stock</t>
+  </si>
+  <si>
+    <t>Id_condicion    FK</t>
+  </si>
+  <si>
+    <t>cond_cancelado</t>
+  </si>
+  <si>
+    <t>usu_nombre</t>
+  </si>
+  <si>
+    <t>acu_parentesco</t>
+  </si>
+  <si>
+    <t>men_valor</t>
+  </si>
+  <si>
+    <t>PQRS_usuasolici</t>
+  </si>
+  <si>
+    <t>nive_imagenEntre</t>
+  </si>
+  <si>
+    <t>hor_nombreEntrenador</t>
+  </si>
+  <si>
+    <t>nove_impuntual</t>
+  </si>
+  <si>
+    <t>imple_precio</t>
+  </si>
+  <si>
+    <t>soli_fecha</t>
+  </si>
+  <si>
+    <t>usu_numdocum</t>
+  </si>
+  <si>
+    <t>men_numRefencia</t>
+  </si>
+  <si>
+    <t>hor_franjas</t>
+  </si>
+  <si>
+    <t>nove_justificado</t>
+  </si>
+  <si>
+    <t>imple_imagen</t>
+  </si>
+  <si>
+    <t>soli_cantidad</t>
+  </si>
+  <si>
+    <t>usu_edad</t>
+  </si>
+  <si>
+    <t>hor_dias</t>
+  </si>
+  <si>
+    <t>imple_observacion</t>
+  </si>
+  <si>
+    <t>soli_talla</t>
+  </si>
+  <si>
+    <t>usu_telefono</t>
+  </si>
+  <si>
+    <t>soli_descripcion</t>
+  </si>
+  <si>
+    <t>usu_fechaNaci</t>
+  </si>
+  <si>
+    <t>soli_comentarios</t>
+  </si>
+  <si>
+    <t>usu_email</t>
+  </si>
+  <si>
+    <t>usu_contraseña</t>
+  </si>
+  <si>
+    <t>usu_cerEPS</t>
+  </si>
+  <si>
+    <t>usu_apellido</t>
+  </si>
+  <si>
+    <t>Gestion de Rendimiento Deportivo</t>
+  </si>
+  <si>
+    <t>TIPO_DOCUMENTO</t>
+  </si>
+  <si>
+    <t>ESTADO_ELEMENTO</t>
+  </si>
+  <si>
+    <t>Id_tipoDoc  PK</t>
+  </si>
+  <si>
+    <t>Id_metodoPago</t>
+  </si>
+  <si>
+    <t>Id_estadoPago PK</t>
+  </si>
+  <si>
+    <t>Id_PQRS  PK</t>
+  </si>
+  <si>
+    <t>Id_tipoPQRS  PK</t>
+  </si>
+  <si>
+    <t>Id_respuesta PK</t>
+  </si>
+  <si>
+    <t>Id_nivel   PK</t>
+  </si>
+  <si>
+    <t>Id_horario   PK</t>
+  </si>
+  <si>
+    <t>Id_horarios         PK</t>
+  </si>
+  <si>
+    <t>Id_horarios   PK</t>
+  </si>
+  <si>
+    <t>Id_usuario FK</t>
+  </si>
+  <si>
+    <t>Id_rendimiento PK</t>
+  </si>
+  <si>
+    <t>Id_asistencia PK</t>
+  </si>
+  <si>
+    <t>Id_novedad  PK</t>
+  </si>
+  <si>
+    <t>Id_implemento     PK</t>
+  </si>
+  <si>
+    <t>Id_estadoImple      PK</t>
+  </si>
+  <si>
+    <t>Id_categoria   PK</t>
+  </si>
+  <si>
+    <t>Id_solicitud   PK</t>
+  </si>
+  <si>
+    <t>Id_condicion   PK</t>
+  </si>
+  <si>
+    <t>tipo_queja</t>
+  </si>
+  <si>
+    <t>Id_PQRS    FK</t>
+  </si>
+  <si>
+    <t>Id_tipo_horario PK</t>
+  </si>
+  <si>
+    <t>dia_nombre     PK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">franja_inicio  </t>
+  </si>
+  <si>
+    <t>Id_asistencia    PKc</t>
+  </si>
+  <si>
+    <t>Id_asistencia  FK</t>
+  </si>
+  <si>
+    <t>Id_estadoImple FK</t>
+  </si>
+  <si>
+    <t>Id_usuario     FK</t>
+  </si>
+  <si>
+    <t>meto_billetera</t>
+  </si>
+  <si>
+    <t>Id_tipoSolicitud  FK</t>
   </si>
   <si>
     <t>cate_descripcion</t>
   </si>
   <si>
-    <t>Id_categoria    FK</t>
-  </si>
-  <si>
-    <t>cond_listoEntrega</t>
-  </si>
-  <si>
-    <t>Id_rol  FK</t>
-  </si>
-  <si>
-    <t>tipo_ti</t>
-  </si>
-  <si>
-    <t>gene_otro</t>
-  </si>
-  <si>
-    <t>rol_atleta</t>
-  </si>
-  <si>
-    <t>acu_apellido</t>
-  </si>
-  <si>
-    <t>Id_estadoPago     FK</t>
-  </si>
-  <si>
-    <t>estaPago_pendiente</t>
-  </si>
-  <si>
-    <t>PQRS_descripcion</t>
-  </si>
-  <si>
-    <t>tipo_sugerencia</t>
-  </si>
-  <si>
-    <t>res_respuesta</t>
-  </si>
-  <si>
-    <t>est_tramite</t>
-  </si>
-  <si>
-    <t>Prio_baja</t>
-  </si>
-  <si>
-    <t>nive_nombre</t>
-  </si>
-  <si>
-    <t>hor_indicaciones</t>
-  </si>
-  <si>
-    <t>franja_fin</t>
-  </si>
-  <si>
-    <t>Tip_Refuerzo</t>
-  </si>
-  <si>
-    <t>ren_descripcionHabilidad</t>
-  </si>
-  <si>
-    <t>asi_justificacion</t>
-  </si>
-  <si>
-    <t>nove_presente</t>
-  </si>
-  <si>
-    <t>imple_nombre</t>
-  </si>
-  <si>
-    <t>Id_implemento   FK</t>
-  </si>
-  <si>
-    <t>cond_entregado</t>
-  </si>
-  <si>
-    <t>Id_nivelClub FK</t>
-  </si>
-  <si>
-    <t>tipo_pasa</t>
-  </si>
-  <si>
-    <t>acu_telefono</t>
-  </si>
-  <si>
-    <t>men_fechaPago</t>
-  </si>
-  <si>
-    <t>PQRS_fechaCrea</t>
-  </si>
-  <si>
-    <t>tipo_solicitud</t>
-  </si>
-  <si>
-    <t>res_fecha</t>
-  </si>
-  <si>
-    <t>Id_PQRS        FK</t>
-  </si>
-  <si>
-    <t>nive_entrenador</t>
-  </si>
-  <si>
-    <t>hor_nombreEntrenador</t>
-  </si>
-  <si>
-    <t>Tip_fisico</t>
-  </si>
-  <si>
-    <t>ren_fecha</t>
-  </si>
-  <si>
-    <t>nove_falta</t>
-  </si>
-  <si>
-    <t>imple_stock</t>
-  </si>
-  <si>
-    <t>Id_condicion    FK</t>
-  </si>
-  <si>
-    <t>cond_cancelado</t>
-  </si>
-  <si>
-    <t>usu_nombre</t>
-  </si>
-  <si>
-    <t>acu_parentesco</t>
-  </si>
-  <si>
-    <t>men_valor</t>
-  </si>
-  <si>
-    <t>PQRS_usuasolici</t>
-  </si>
-  <si>
-    <t>nive_imagenEntre</t>
-  </si>
-  <si>
-    <t>hor_franjas</t>
-  </si>
-  <si>
-    <t>nove_impuntual</t>
-  </si>
-  <si>
-    <t>imple_precio</t>
-  </si>
-  <si>
-    <t>soli_fecha</t>
-  </si>
-  <si>
-    <t>usu_numdocum</t>
-  </si>
-  <si>
-    <t>men_numRefencia</t>
-  </si>
-  <si>
-    <t>hor_dias</t>
-  </si>
-  <si>
-    <t>nove_justificado</t>
-  </si>
-  <si>
-    <t>imple_imagen</t>
-  </si>
-  <si>
-    <t>soli_cantidad</t>
-  </si>
-  <si>
-    <t>usu_edad</t>
-  </si>
-  <si>
-    <t>imple_observacion</t>
-  </si>
-  <si>
-    <t>soli_talla</t>
-  </si>
-  <si>
-    <t>usu_telefono</t>
-  </si>
-  <si>
-    <t>imple_talla</t>
-  </si>
-  <si>
-    <t>soli_descripcion</t>
-  </si>
-  <si>
-    <t>usu_fechaNaci</t>
-  </si>
-  <si>
-    <t>soli_comentarios</t>
-  </si>
-  <si>
-    <t>usu_email</t>
-  </si>
-  <si>
-    <t>usu_contraseña</t>
-  </si>
-  <si>
-    <t>usu_cerEPS</t>
-  </si>
-  <si>
-    <t>usu_apellido</t>
-  </si>
-  <si>
-    <t>Gestion de Rendimiento Deportivo</t>
-  </si>
-  <si>
-    <t>TIPO_DOCUMENTO</t>
-  </si>
-  <si>
-    <t>ESTADO_ELEMENTO</t>
-  </si>
-  <si>
-    <t>Id_tipoDoc  PK</t>
-  </si>
-  <si>
-    <t>Id_metodoPago</t>
-  </si>
-  <si>
-    <t>Id_estadoPago PK</t>
-  </si>
-  <si>
-    <t>Id_PQRS  PK</t>
-  </si>
-  <si>
-    <t>Id_tipoSolicitud  PK</t>
-  </si>
-  <si>
-    <t>Id_respuesta PK</t>
-  </si>
-  <si>
-    <t>Id_nivel   PK</t>
-  </si>
-  <si>
-    <t>Id_horario   PK</t>
-  </si>
-  <si>
-    <t>Id_horario         PKc</t>
-  </si>
-  <si>
-    <t>Id_horario   PKc</t>
-  </si>
-  <si>
-    <t>Id_usuario FK</t>
-  </si>
-  <si>
-    <t>Id_rendimiento PK</t>
-  </si>
-  <si>
-    <t>Id_asistencia PK</t>
-  </si>
-  <si>
-    <t>Id_novedad  PK</t>
-  </si>
-  <si>
-    <t>Id_elemento     PK</t>
-  </si>
-  <si>
-    <t>Id_estadoElem      PK</t>
-  </si>
-  <si>
-    <t>Id_categoria   PK</t>
-  </si>
-  <si>
-    <t>Id_solicitud   PK</t>
-  </si>
-  <si>
-    <t>Id_condicion   PK</t>
-  </si>
-  <si>
-    <t>Id_tipoDoc FK</t>
-  </si>
-  <si>
-    <t>tipo_queja</t>
-  </si>
-  <si>
-    <t>Id_PQRS    FK</t>
-  </si>
-  <si>
-    <t>Id_usuario (entrenador)  FK</t>
-  </si>
-  <si>
-    <t>Id_nivel        FK</t>
-  </si>
-  <si>
-    <t>dia_nombre     PKc</t>
-  </si>
-  <si>
-    <t>franja_inicio  PKc</t>
-  </si>
-  <si>
-    <t>Id_asistencia    PKc</t>
-  </si>
-  <si>
-    <t>Id_asistencia  FK</t>
-  </si>
-  <si>
-    <t>Id_estadoElem FK</t>
-  </si>
-  <si>
-    <t>Id_usuario     FK</t>
-  </si>
-  <si>
-    <t>meto_billetera</t>
-  </si>
-  <si>
-    <t>Id_tipoSolicitud  FK</t>
-  </si>
-  <si>
-    <t>nive_nivel</t>
+    <t>Id_categoria FK</t>
   </si>
   <si>
     <t>hor_nombre</t>
   </si>
   <si>
-    <t>Id_categoria FK</t>
-  </si>
-  <si>
-    <t>nive_descripcion</t>
-  </si>
-  <si>
-    <t>Id_elemento FK</t>
+    <t>Id_implemento FK</t>
+  </si>
+  <si>
+    <t>Id_PQRS  FK</t>
   </si>
   <si>
     <t>Id_condicion  FK</t>
@@ -668,21 +659,9 @@
     <t>usu_numDocumento</t>
   </si>
   <si>
-    <t>ele_precio</t>
-  </si>
-  <si>
-    <t>ele_imagen</t>
-  </si>
-  <si>
-    <t>ele_observacion</t>
-  </si>
-  <si>
     <t>usu_nivel</t>
   </si>
   <si>
-    <t>ele_talla</t>
-  </si>
-  <si>
     <t>TIPO_HORARIO</t>
   </si>
   <si>
@@ -692,25 +671,25 @@
     <t>IMPLEMENTO_TALLAS</t>
   </si>
   <si>
-    <t>Id_horario         FK</t>
+    <t>Id_tipoPQRS PK</t>
+  </si>
+  <si>
+    <t>Id_niveles   PK</t>
+  </si>
+  <si>
+    <t>Id_horarios         FK</t>
   </si>
   <si>
     <t>Id_horario   FK</t>
   </si>
   <si>
-    <t>Id_tipo_horario PK</t>
+    <t xml:space="preserve">Id_asistencia </t>
   </si>
   <si>
     <t>Id_tipoNovedad PK</t>
   </si>
   <si>
-    <t>Id_implemento     PK</t>
-  </si>
-  <si>
     <t>Id_talla         PK</t>
-  </si>
-  <si>
-    <t>Id_estadoImple      PK</t>
   </si>
   <si>
     <r>
@@ -719,7 +698,7 @@
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t>tipo_nombre</t>
+      <t>tipodoc_nombre</t>
     </r>
     <r>
       <rPr>
@@ -858,27 +837,25 @@
     <t xml:space="preserve">dia_nombre     </t>
   </si>
   <si>
-    <t xml:space="preserve">franja_inicio  </t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Calibri"/>
-        <b/>
         <color theme="1"/>
         <sz val="11.0"/>
       </rPr>
-      <t xml:space="preserve">tipo_nombre </t>
+      <t xml:space="preserve">Tip_nombre </t>
     </r>
     <r>
       <rPr>
         <rFont val="Calibri"/>
-        <b/>
         <color theme="1"/>
         <sz val="9.0"/>
       </rPr>
       <t>(Partner / Competencia / Refuerzo / Físico)</t>
     </r>
+  </si>
+  <si>
+    <t>asi_fechaAsis  FK</t>
   </si>
   <si>
     <r>
@@ -899,9 +876,6 @@
     </r>
   </si>
   <si>
-    <t>Id_estadoImple FK</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Calibri"/>
@@ -938,9 +912,6 @@
     </r>
   </si>
   <si>
-    <t>Id_implemento FK</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <rFont val="Calibri"/>
@@ -959,32 +930,62 @@
     </r>
   </si>
   <si>
-    <t>id_tipo_horario  FK</t>
+    <t>Id_tipoPQRS  FK</t>
+  </si>
+  <si>
+    <t>nive_nivel</t>
+  </si>
+  <si>
+    <t>Id_tipoHorario  FK</t>
   </si>
   <si>
     <t>Id_horarioDia      PK</t>
   </si>
   <si>
+    <t>asi_fechaAsis  PK</t>
+  </si>
+  <si>
     <t>Id_tipoNovedad FK</t>
   </si>
   <si>
-    <t>Id_horarioFran    PK</t>
-  </si>
-  <si>
-    <t>Id_nivel FK</t>
+    <t>Id_implemento  FK</t>
+  </si>
+  <si>
+    <t>nive_descripcion</t>
+  </si>
+  <si>
+    <t>Id_franja    PK</t>
+  </si>
+  <si>
+    <t>Id_niveles FK</t>
+  </si>
+  <si>
+    <t>Id_novedad  FK</t>
+  </si>
+  <si>
+    <t>nove_nombre</t>
   </si>
   <si>
     <t>Id_prioridad   FK</t>
   </si>
   <si>
     <t>Id_talla         FK</t>
+  </si>
+  <si>
+    <t>imple_observaciones</t>
+  </si>
+  <si>
+    <t>Id_condicion FK</t>
+  </si>
+  <si>
+    <t>Id_solicitud   FK</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1002,17 +1003,26 @@
       <b/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1125,7 +1135,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="52">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1141,7 +1151,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="4" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="1" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
@@ -1149,9 +1159,6 @@
     </xf>
     <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="4" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -1161,56 +1168,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+    <xf borderId="4" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="4" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="4" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="3" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1221,7 +1205,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf borderId="1" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -1229,50 +1213,46 @@
     <xf borderId="4" fillId="2" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf borderId="4" fillId="4" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="7" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="4" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="4" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="5" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="4" fillId="7" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="4" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1614,7 +1594,7 @@
       <c r="B4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>6</v>
       </c>
       <c r="F4" s="9" t="s">
@@ -1623,571 +1603,568 @@
       <c r="H4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="11"/>
+      <c r="I4" s="10"/>
       <c r="J4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="12"/>
+      <c r="K4" s="11"/>
       <c r="L4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="12"/>
+      <c r="M4" s="11"/>
       <c r="N4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="12"/>
+      <c r="O4" s="11"/>
       <c r="P4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="R4" s="13" t="s">
+      <c r="R4" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="13" t="s">
+      <c r="T4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="V4" s="13" t="s">
+      <c r="V4" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="X4" s="14" t="s">
+      <c r="X4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="Z4" s="14" t="s">
+      <c r="Z4" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="AB4" s="15" t="s">
+      <c r="AB4" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="AD4" s="15" t="s">
+      <c r="AD4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="AF4" s="15" t="s">
+      <c r="AF4" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="AH4" s="15" t="s">
+      <c r="AH4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="AJ4" s="16" t="s">
+      <c r="AJ4" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="AL4" s="17" t="s">
+      <c r="AL4" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="AM4" s="18"/>
-      <c r="AN4" s="19" t="s">
+      <c r="AM4" s="11"/>
+      <c r="AN4" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="AP4" s="19" t="s">
+      <c r="AP4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="AR4" s="20" t="s">
+      <c r="AR4" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="AT4" s="21" t="s">
+      <c r="AT4" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="AV4" s="20" t="s">
+      <c r="AV4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="AX4" s="20" t="s">
+      <c r="AX4" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="AZ4" s="20" t="s">
+      <c r="AZ4" s="17" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="22" t="s">
+      <c r="F5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="22" t="s">
+      <c r="I5" s="20"/>
+      <c r="J5" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="K5" s="24"/>
-      <c r="L5" s="22" t="s">
+      <c r="K5" s="21"/>
+      <c r="L5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="24"/>
-      <c r="N5" s="22" t="s">
+      <c r="M5" s="21"/>
+      <c r="N5" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O5" s="24"/>
-      <c r="P5" s="22" t="s">
+      <c r="O5" s="21"/>
+      <c r="P5" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="R5" s="22" t="s">
+      <c r="R5" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="T5" s="22" t="s">
+      <c r="T5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="V5" s="22" t="s">
+      <c r="V5" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="X5" s="25" t="s">
+      <c r="X5" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="Z5" s="25" t="s">
+      <c r="Z5" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="AB5" s="22" t="s">
+      <c r="AB5" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="AD5" s="22" t="s">
+      <c r="AD5" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="AF5" s="22" t="s">
+      <c r="AF5" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="AH5" s="22" t="s">
+      <c r="AH5" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="AJ5" s="22" t="s">
+      <c r="AJ5" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="AL5" s="25" t="s">
+      <c r="AL5" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="AM5" s="18"/>
-      <c r="AN5" s="22" t="s">
+      <c r="AM5" s="11"/>
+      <c r="AN5" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="AP5" s="22" t="s">
+      <c r="AP5" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="AR5" s="22" t="s">
+      <c r="AR5" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="AT5" s="22" t="s">
+      <c r="AT5" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="AV5" s="22" t="s">
+      <c r="AV5" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="AX5" s="22" t="s">
+      <c r="AX5" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="AZ5" s="22" t="s">
+      <c r="AZ5" s="18" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="23" t="s">
         <v>58</v>
       </c>
-      <c r="F6" s="27" t="s">
+      <c r="F6" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="H6" s="26" t="s">
+      <c r="H6" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="I6" s="28"/>
-      <c r="J6" s="22" t="s">
+      <c r="I6" s="20"/>
+      <c r="J6" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="K6" s="24"/>
-      <c r="L6" s="22" t="s">
+      <c r="K6" s="21"/>
+      <c r="L6" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="24"/>
-      <c r="N6" s="26" t="s">
+      <c r="M6" s="21"/>
+      <c r="N6" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="26" t="s">
+      <c r="O6" s="21"/>
+      <c r="P6" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="R6" s="22" t="s">
+      <c r="R6" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="T6" s="27" t="s">
+      <c r="T6" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="V6" s="22" t="s">
+      <c r="V6" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="X6" s="29" t="s">
+      <c r="X6" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="Z6" s="29" t="s">
+      <c r="Z6" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="AB6" s="22" t="s">
+      <c r="AB6" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="AD6" s="22" t="s">
+      <c r="AD6" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="AF6" s="22" t="s">
+      <c r="AF6" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="AH6" s="22" t="s">
+      <c r="AH6" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="AJ6" s="27" t="s">
+      <c r="AJ6" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="AL6" s="25" t="s">
+      <c r="AL6" s="22" t="s">
         <v>75</v>
       </c>
-      <c r="AM6" s="18"/>
-      <c r="AN6" s="22" t="s">
+      <c r="AM6" s="11"/>
+      <c r="AN6" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="AP6" s="22" t="s">
+      <c r="AP6" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="AR6" s="22" t="s">
+      <c r="AR6" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="AT6" s="26" t="s">
+      <c r="AT6" s="23" t="s">
         <v>79</v>
       </c>
-      <c r="AV6" s="26" t="s">
+      <c r="AV6" s="23" t="s">
         <v>80</v>
       </c>
-      <c r="AX6" s="22" t="s">
+      <c r="AX6" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="AZ6" s="26" t="s">
+      <c r="AZ6" s="23" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="I7" s="28"/>
-      <c r="J7" s="26" t="s">
+      <c r="I7" s="20"/>
+      <c r="J7" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="22" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="M7" s="12"/>
-      <c r="N7" s="27" t="s">
+      <c r="M7" s="11"/>
+      <c r="N7" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="O7" s="12"/>
-      <c r="P7" s="26" t="s">
+      <c r="O7" s="11"/>
+      <c r="P7" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="R7" s="22" t="s">
+      <c r="R7" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="T7" s="26" t="s">
+      <c r="T7" s="23" t="s">
         <v>92</v>
       </c>
-      <c r="V7" s="22" t="s">
+      <c r="V7" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="X7" s="29" t="s">
+      <c r="X7" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="Z7" s="29" t="s">
+      <c r="Z7" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="AB7" s="27" t="s">
+      <c r="AB7" s="23" t="s">
         <v>96</v>
       </c>
-      <c r="AD7" s="27" t="s">
+      <c r="AD7" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="AF7" s="26" t="s">
+      <c r="AF7" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="AH7" s="26" t="s">
+      <c r="AH7" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="AJ7" s="27" t="s">
+      <c r="AJ7" s="23" t="s">
         <v>100</v>
       </c>
-      <c r="AL7" s="29" t="s">
+      <c r="AL7" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="AM7" s="18"/>
-      <c r="AN7" s="26" t="s">
+      <c r="AM7" s="11"/>
+      <c r="AN7" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="AP7" s="22" t="s">
+      <c r="AP7" s="18" t="s">
         <v>103</v>
       </c>
-      <c r="AR7" s="22" t="s">
+      <c r="AR7" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="AT7" s="26" t="s">
+      <c r="AT7" s="23" t="s">
         <v>105</v>
       </c>
-      <c r="AV7" s="26" t="s">
+      <c r="AX7" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="AX7" s="22" t="s">
+      <c r="AZ7" s="23" t="s">
         <v>107</v>
-      </c>
-      <c r="AZ7" s="26" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="F8" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="H8" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="H8" s="26" t="s">
+      <c r="I8" s="20"/>
+      <c r="J8" s="23" t="s">
         <v>112</v>
       </c>
-      <c r="I8" s="28"/>
-      <c r="J8" s="27" t="s">
+      <c r="K8" s="11"/>
+      <c r="L8" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="K8" s="12"/>
-      <c r="L8" s="22" t="s">
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="27" t="s">
+      <c r="R8" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="R8" s="26" t="s">
+      <c r="T8" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="T8" s="26" t="s">
+      <c r="V8" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="V8" s="26" t="s">
+      <c r="X8" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="X8" s="29" t="s">
+      <c r="Z8" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="Z8" s="29" t="s">
+      <c r="AB8" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="AB8" s="27" t="s">
+      <c r="AD8" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="AD8" s="27" t="s">
+      <c r="AH8" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="AH8" s="26" t="s">
+      <c r="AJ8" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="AJ8" s="29" t="s">
+      <c r="AL8" s="24" t="s">
         <v>124</v>
       </c>
-      <c r="AL8" s="29" t="s">
+      <c r="AM8" s="11"/>
+      <c r="AN8" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="AM8" s="18"/>
-      <c r="AN8" s="26" t="s">
+      <c r="AP8" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="AP8" s="26" t="s">
+      <c r="AR8" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="AR8" s="27" t="s">
+      <c r="AX8" s="18" t="s">
         <v>128</v>
       </c>
-      <c r="AX8" s="22" t="s">
+      <c r="AZ8" s="23" t="s">
         <v>129</v>
-      </c>
-      <c r="AZ8" s="26" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>131</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="J9" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="J9" s="26" t="s">
+      <c r="K9" s="11"/>
+      <c r="L9" s="23" t="s">
         <v>133</v>
       </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="26" t="s">
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="R9" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="R9" s="26" t="s">
+      <c r="T9" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="T9" s="26" t="s">
+      <c r="V9" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="V9" s="26" t="s">
+      <c r="X9" s="18" t="s">
         <v>137</v>
       </c>
-      <c r="X9" s="22" t="s">
+      <c r="Z9" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="AB9" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="Z9" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="AB9" s="27" t="s">
+      <c r="AD9" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="AD9" s="27" t="s">
+      <c r="AJ9" s="24" t="s">
         <v>140</v>
       </c>
-      <c r="AJ9" s="29" t="s">
+      <c r="AL9" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="AL9" s="29" t="s">
+      <c r="AM9" s="11"/>
+      <c r="AP9" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AM9" s="18"/>
-      <c r="AP9" s="26" t="s">
+      <c r="AR9" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AR9" s="27" t="s">
+      <c r="AX9" s="18" t="s">
         <v>144</v>
       </c>
-      <c r="AX9" s="22" t="s">
+      <c r="AZ9" s="23" t="s">
         <v>145</v>
-      </c>
-      <c r="AZ9" s="26" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10" s="26"/>
+      <c r="J10" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="D10" s="31"/>
-      <c r="J10" s="26" t="s">
+      <c r="L10" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="L10" s="26" t="s">
+      <c r="R10" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="R10" s="27" t="s">
+      <c r="AB10" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="AB10" s="27" t="s">
+      <c r="AD10" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="AD10" s="27" t="s">
+      <c r="AM10" s="11"/>
+      <c r="AP10" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="AM10" s="18"/>
-      <c r="AP10" s="26" t="s">
+      <c r="AR10" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="AR10" s="27" t="s">
+      <c r="AX10" s="23" t="s">
         <v>154</v>
-      </c>
-      <c r="AX10" s="26" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="23" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="E11" s="27"/>
+      <c r="L11" s="23" t="s">
         <v>156</v>
       </c>
-      <c r="D11" s="32"/>
-      <c r="E11" s="33"/>
-      <c r="L11" s="27" t="s">
+      <c r="AD11" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="AD11" s="27" t="s">
+      <c r="AM11" s="11"/>
+      <c r="AP11" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="AM11" s="18"/>
-      <c r="AP11" s="26" t="s">
+      <c r="AR11" s="23" t="s">
         <v>159</v>
       </c>
-      <c r="AR11" s="27" t="s">
+      <c r="AX11" s="23" t="s">
         <v>160</v>
-      </c>
-      <c r="AX11" s="26" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="23" t="s">
+        <v>161</v>
+      </c>
+      <c r="AD12" s="23" t="s">
         <v>162</v>
       </c>
-      <c r="AM12" s="18"/>
-      <c r="AR12" s="27" t="s">
+      <c r="AM12" s="11"/>
+      <c r="AR12" s="23" t="s">
         <v>163</v>
       </c>
-      <c r="AX12" s="26" t="s">
+      <c r="AX12" s="23" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="AM13" s="18"/>
-      <c r="AR13" s="29" t="s">
+      <c r="AM13" s="11"/>
+      <c r="AX13" s="23" t="s">
         <v>166</v>
-      </c>
-      <c r="AX13" s="26" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="AX14" s="24" t="s">
         <v>168</v>
-      </c>
-      <c r="AX14" s="29" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="T15" s="12"/>
+      <c r="B15" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="T15" s="11"/>
     </row>
     <row r="16">
-      <c r="B16" s="26" t="s">
-        <v>171</v>
+      <c r="B16" s="23" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="27" t="s">
-        <v>172</v>
+      <c r="B17" s="23" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="29" t="s">
-        <v>173</v>
+      <c r="B18" s="24" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -3172,11 +3149,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="B2:P2"/>
     <mergeCell ref="R2:Z2"/>
     <mergeCell ref="AB2:AJ2"/>
     <mergeCell ref="AL2:AP2"/>
     <mergeCell ref="AR2:AZ2"/>
-    <mergeCell ref="B2:P2"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -3219,7 +3196,7 @@
     <col customWidth="1" min="25" max="25" width="10.71"/>
     <col customWidth="1" min="26" max="26" width="25.0"/>
     <col customWidth="1" min="27" max="27" width="10.71"/>
-    <col customWidth="1" min="28" max="28" width="17.0"/>
+    <col customWidth="1" min="28" max="28" width="19.14"/>
     <col customWidth="1" min="29" max="29" width="10.71"/>
     <col customWidth="1" min="30" max="30" width="24.43"/>
     <col customWidth="1" min="31" max="31" width="10.71"/>
@@ -3233,13 +3210,13 @@
     <col customWidth="1" min="39" max="39" width="10.71"/>
     <col customWidth="1" min="40" max="40" width="19.14"/>
     <col customWidth="1" min="41" max="41" width="10.71"/>
-    <col customWidth="1" min="42" max="42" width="19.29"/>
+    <col customWidth="1" min="42" max="42" width="20.43"/>
     <col customWidth="1" min="43" max="43" width="10.71"/>
     <col customWidth="1" min="44" max="44" width="22.0"/>
     <col customWidth="1" min="45" max="45" width="10.71"/>
     <col customWidth="1" min="46" max="46" width="16.43"/>
     <col customWidth="1" min="47" max="47" width="10.71"/>
-    <col customWidth="1" min="48" max="48" width="15.57"/>
+    <col customWidth="1" min="48" max="48" width="18.0"/>
     <col customWidth="1" min="49" max="49" width="10.71"/>
     <col customWidth="1" min="50" max="50" width="18.71"/>
     <col customWidth="1" min="51" max="51" width="10.71"/>
@@ -3263,7 +3240,7 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3"/>
-      <c r="R2" s="34" t="s">
+      <c r="R2" s="28" t="s">
         <v>1</v>
       </c>
       <c r="S2" s="2"/>
@@ -3272,7 +3249,7 @@
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
       <c r="X2" s="3"/>
-      <c r="Z2" s="35" t="s">
+      <c r="Z2" s="29" t="s">
         <v>2</v>
       </c>
       <c r="AA2" s="2"/>
@@ -3283,14 +3260,14 @@
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
       <c r="AH2" s="3"/>
-      <c r="AJ2" s="36" t="s">
-        <v>174</v>
+      <c r="AJ2" s="30" t="s">
+        <v>173</v>
       </c>
       <c r="AK2" s="2"/>
       <c r="AL2" s="2"/>
       <c r="AM2" s="2"/>
       <c r="AN2" s="3"/>
-      <c r="AP2" s="37" t="s">
+      <c r="AP2" s="31" t="s">
         <v>4</v>
       </c>
       <c r="AQ2" s="2"/>
@@ -3303,519 +3280,531 @@
       <c r="AX2" s="3"/>
     </row>
     <row r="4">
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="F4" s="32" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>9</v>
+      </c>
+      <c r="K4" s="11"/>
+      <c r="L4" s="32" t="s">
+        <v>10</v>
+      </c>
+      <c r="M4" s="11"/>
+      <c r="N4" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="O4" s="11"/>
+      <c r="P4" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="R4" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="T4" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="V4" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="X4" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="Z4" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="AB4" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD4" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="AF4" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG4" s="11"/>
+      <c r="AH4" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ4" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="AL4" s="36" t="s">
+        <v>24</v>
+      </c>
+      <c r="AN4" s="36" t="s">
+        <v>25</v>
+      </c>
+      <c r="AP4" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="AR4" s="37" t="s">
         <v>175</v>
       </c>
-      <c r="F4" s="38" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="38" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" s="38" t="s">
-        <v>9</v>
-      </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="38" t="s">
-        <v>10</v>
-      </c>
-      <c r="M4" s="12"/>
-      <c r="N4" s="38" t="s">
-        <v>11</v>
-      </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="38" t="s">
-        <v>12</v>
-      </c>
-      <c r="R4" s="39" t="s">
-        <v>13</v>
-      </c>
-      <c r="T4" s="39" t="s">
-        <v>14</v>
-      </c>
-      <c r="V4" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="X4" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z4" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="AB4" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="AD4" s="41" t="s">
-        <v>20</v>
-      </c>
-      <c r="AF4" s="41" t="s">
-        <v>21</v>
-      </c>
-      <c r="AG4" s="12"/>
-      <c r="AH4" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="AJ4" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="AL4" s="42" t="s">
-        <v>24</v>
-      </c>
-      <c r="AN4" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="AP4" s="43" t="s">
-        <v>26</v>
-      </c>
-      <c r="AR4" s="43" t="s">
-        <v>176</v>
-      </c>
-      <c r="AT4" s="43" t="s">
+      <c r="AT4" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="AV4" s="43" t="s">
+      <c r="AV4" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="AX4" s="43" t="s">
+      <c r="AX4" s="37" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D5" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="H5" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="K5" s="21"/>
+      <c r="L5" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M5" s="21"/>
+      <c r="N5" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="F5" s="44" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="24"/>
-      <c r="L5" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="M5" s="24"/>
-      <c r="N5" s="44" t="s">
+      <c r="O5" s="21"/>
+      <c r="P5" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="O5" s="24"/>
-      <c r="P5" s="44" t="s">
+      <c r="R5" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="R5" s="44" t="s">
+      <c r="T5" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="T5" s="44" t="s">
+      <c r="V5" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="V5" s="44" t="s">
+      <c r="X5" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="Z5" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="X5" s="25" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z5" s="44" t="s">
+      <c r="AB5" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="AB5" s="44" t="s">
+      <c r="AD5" s="19" t="s">
         <v>184</v>
       </c>
-      <c r="AD5" s="44" t="s">
+      <c r="AF5" s="19" t="s">
         <v>185</v>
       </c>
-      <c r="AF5" s="44" t="s">
+      <c r="AG5" s="21"/>
+      <c r="AH5" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="AG5" s="24"/>
-      <c r="AH5" s="44" t="s">
+      <c r="AJ5" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="AJ5" s="25" t="s">
+      <c r="AL5" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="AL5" s="22" t="s">
+      <c r="AN5" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="AN5" s="22" t="s">
+      <c r="AP5" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="AP5" s="44" t="s">
+      <c r="AR5" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="AR5" s="44" t="s">
+      <c r="AT5" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="AT5" s="44" t="s">
+      <c r="AV5" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="AV5" s="44" t="s">
+      <c r="AX5" s="18" t="s">
         <v>194</v>
-      </c>
-      <c r="AX5" s="44" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="F6" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K6" s="21"/>
+      <c r="L6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="21"/>
+      <c r="N6" s="23" t="s">
+        <v>63</v>
+      </c>
+      <c r="O6" s="21"/>
+      <c r="P6" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="R6" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="T6" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="V6" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="F6" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="H6" s="26" t="s">
-        <v>60</v>
-      </c>
-      <c r="J6" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="K6" s="24"/>
-      <c r="L6" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" s="24"/>
-      <c r="N6" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="26" t="s">
-        <v>64</v>
-      </c>
-      <c r="R6" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="T6" s="26" t="s">
+      <c r="X6" s="24" t="s">
+        <v>69</v>
+      </c>
+      <c r="Z6" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB6" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="V6" s="44" t="s">
+      <c r="AD6" s="38" t="s">
         <v>198</v>
       </c>
-      <c r="X6" s="29" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z6" s="44" t="s">
+      <c r="AF6" s="38" t="s">
         <v>199</v>
       </c>
-      <c r="AB6" s="44" t="s">
+      <c r="AG6" s="21"/>
+      <c r="AH6" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="AD6" s="26" t="s">
+      <c r="AJ6" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="AL6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="AN6" s="39" t="s">
         <v>201</v>
       </c>
-      <c r="AF6" s="22" t="s">
+      <c r="AP6" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="AG6" s="24"/>
-      <c r="AH6" s="22" t="s">
+      <c r="AR6" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="AT6" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="AV6" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="AJ6" s="25" t="s">
-        <v>187</v>
-      </c>
-      <c r="AL6" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="AN6" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="AP6" s="44" t="s">
-        <v>205</v>
-      </c>
-      <c r="AR6" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="AT6" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="AV6" s="44" t="s">
-        <v>206</v>
-      </c>
-      <c r="AX6" s="26" t="s">
+      <c r="AX6" s="23" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="F7" s="27" t="s">
+      <c r="F7" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="H7" s="26" t="s">
+      <c r="H7" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="J7" s="26" t="s">
+      <c r="J7" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="22" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="M7" s="12"/>
-      <c r="N7" s="26" t="s">
+      <c r="M7" s="11"/>
+      <c r="N7" s="23" t="s">
+        <v>204</v>
+      </c>
+      <c r="O7" s="11"/>
+      <c r="P7" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="R7" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="T7" s="23" t="s">
+        <v>92</v>
+      </c>
+      <c r="V7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="X7" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="Z7" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB7" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF7" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="AG7" s="11"/>
+      <c r="AH7" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="AJ7" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="AL7" s="23" t="s">
+        <v>102</v>
+      </c>
+      <c r="AN7" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="AP7" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="AR7" s="23" t="s">
+        <v>105</v>
+      </c>
+      <c r="AT7" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="AV7" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="O7" s="12"/>
-      <c r="P7" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="R7" s="44" t="s">
-        <v>208</v>
-      </c>
-      <c r="T7" s="26" t="s">
-        <v>92</v>
-      </c>
-      <c r="V7" s="44" t="s">
-        <v>77</v>
-      </c>
-      <c r="X7" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="Z7" s="26" t="s">
-        <v>209</v>
-      </c>
-      <c r="AB7" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="AF7" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG7" s="12"/>
-      <c r="AH7" s="26" t="s">
-        <v>127</v>
-      </c>
-      <c r="AJ7" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="AL7" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="AN7" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="AP7" s="44" t="s">
-        <v>65</v>
-      </c>
-      <c r="AR7" s="26" t="s">
-        <v>105</v>
-      </c>
-      <c r="AT7" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="AV7" s="44" t="s">
-        <v>211</v>
-      </c>
-      <c r="AX7" s="26" t="s">
-        <v>108</v>
+      <c r="AX7" s="23" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="44" t="s">
+      <c r="B8" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>109</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="F8" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="F8" s="26" t="s">
+      <c r="H8" s="23" t="s">
         <v>111</v>
       </c>
-      <c r="H8" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="J8" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="K8" s="12"/>
-      <c r="L8" s="22" t="s">
+      <c r="J8" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="23" t="s">
         <v>114</v>
       </c>
-      <c r="M8" s="12"/>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="27" t="s">
+      <c r="R8" s="23" t="s">
         <v>115</v>
       </c>
-      <c r="R8" s="26" t="s">
+      <c r="T8" s="23" t="s">
         <v>116</v>
       </c>
-      <c r="T8" s="26" t="s">
+      <c r="V8" s="23" t="s">
         <v>117</v>
       </c>
-      <c r="V8" s="26" t="s">
-        <v>118</v>
-      </c>
-      <c r="X8" s="29" t="s">
+      <c r="X8" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="Z8" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="Z8" s="26" t="s">
-        <v>212</v>
-      </c>
-      <c r="AG8" s="12"/>
-      <c r="AH8" s="26" t="s">
-        <v>143</v>
-      </c>
-      <c r="AJ8" s="29" t="s">
+      <c r="AB8" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="AG8" s="11"/>
+      <c r="AH8" s="23" t="s">
+        <v>142</v>
+      </c>
+      <c r="AJ8" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="AL8" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="AL8" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="AN8" s="46" t="s">
-        <v>153</v>
-      </c>
-      <c r="AP8" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="AV8" s="44" t="s">
-        <v>213</v>
-      </c>
-      <c r="AX8" s="26" t="s">
-        <v>130</v>
+      <c r="AN8" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="AP8" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="AV8" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="AX8" s="23" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="J9" s="23" t="s">
         <v>147</v>
       </c>
-      <c r="D9" s="30" t="s">
-        <v>132</v>
-      </c>
-      <c r="J9" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="26" t="s">
+      <c r="K9" s="11"/>
+      <c r="L9" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
+      <c r="R9" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="M9" s="12"/>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="R9" s="26" t="s">
+      <c r="T9" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="T9" s="26" t="s">
+      <c r="V9" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="V9" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="AH9" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="AJ9" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="AN9" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="AP9" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="AV9" s="44" t="s">
-        <v>214</v>
-      </c>
-      <c r="AX9" s="26" t="s">
-        <v>146</v>
+      <c r="X9" s="19" t="s">
+        <v>210</v>
+      </c>
+      <c r="Z9" s="41" t="s">
+        <v>138</v>
+      </c>
+      <c r="AH9" s="23" t="s">
+        <v>152</v>
+      </c>
+      <c r="AJ9" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="AN9" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="AP9" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="AV9" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="AX9" s="23" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="26" t="s">
-        <v>215</v>
-      </c>
-      <c r="D10" s="31"/>
-      <c r="L10" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="AH10" s="26" t="s">
-        <v>159</v>
-      </c>
-      <c r="AN10" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="AP10" s="26" t="s">
-        <v>216</v>
-      </c>
-      <c r="AV10" s="26" t="s">
-        <v>155</v>
+      <c r="B10" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10" s="26"/>
+      <c r="L10" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="Z10" s="41" t="s">
+        <v>150</v>
+      </c>
+      <c r="AH10" s="23" t="s">
+        <v>158</v>
+      </c>
+      <c r="AN10" s="23" t="s">
+        <v>126</v>
+      </c>
+      <c r="AP10" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="AV10" s="23" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="26" t="s">
-        <v>162</v>
-      </c>
-      <c r="D11" s="32"/>
-      <c r="L11" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="AP11" s="26" t="s">
-        <v>217</v>
-      </c>
-      <c r="AV11" s="26" t="s">
-        <v>161</v>
+      <c r="B11" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="L11" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="AP11" s="38" t="s">
+        <v>159</v>
+      </c>
+      <c r="AV11" s="23" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="AH12" s="12"/>
-      <c r="AP12" s="26" t="s">
-        <v>218</v>
-      </c>
-      <c r="AV12" s="26" t="s">
-        <v>167</v>
+      <c r="AH12" s="11"/>
+      <c r="AP12" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="AV12" s="23" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="26" t="s">
-        <v>219</v>
-      </c>
-      <c r="AP13" s="26" t="s">
-        <v>220</v>
-      </c>
-      <c r="AV13" s="29" t="s">
-        <v>169</v>
+      <c r="B13" s="23" t="s">
+        <v>213</v>
+      </c>
+      <c r="AV13" s="24" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="26" t="s">
-        <v>168</v>
+      <c r="B14" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="AV14" s="23" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="T15" s="12"/>
+      <c r="B15" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="T15" s="11"/>
     </row>
     <row r="16">
-      <c r="B16" s="26" t="s">
-        <v>171</v>
+      <c r="B16" s="23" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="29" t="s">
-        <v>173</v>
+      <c r="B17" s="24" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="27" t="s">
-        <v>172</v>
+      <c r="B18" s="23" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -4800,11 +4789,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="B2:P2"/>
     <mergeCell ref="R2:X2"/>
     <mergeCell ref="Z2:AH2"/>
     <mergeCell ref="AJ2:AN2"/>
     <mergeCell ref="AP2:AX2"/>
-    <mergeCell ref="B2:P2"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -4823,7 +4812,7 @@
     <col customWidth="1" min="1" max="1" width="10.71"/>
     <col customWidth="1" min="2" max="2" width="21.86"/>
     <col customWidth="1" min="3" max="3" width="10.71"/>
-    <col customWidth="1" min="4" max="4" width="28.14"/>
+    <col customWidth="1" min="4" max="4" width="30.29"/>
     <col customWidth="1" min="5" max="5" width="10.71"/>
     <col customWidth="1" min="6" max="6" width="32.29"/>
     <col customWidth="1" min="7" max="7" width="10.71"/>
@@ -4862,10 +4851,10 @@
     <col customWidth="1" min="40" max="40" width="16.43"/>
     <col customWidth="1" min="41" max="41" width="8.86"/>
     <col customWidth="1" min="42" max="42" width="19.29"/>
-    <col customWidth="1" min="43" max="43" width="11.14"/>
-    <col customWidth="1" min="44" max="44" width="46.71"/>
+    <col customWidth="1" min="43" max="43" width="12.57"/>
+    <col customWidth="1" min="44" max="44" width="43.86"/>
     <col customWidth="1" min="45" max="45" width="12.57"/>
-    <col customWidth="1" min="46" max="46" width="19.29"/>
+    <col customWidth="1" min="46" max="46" width="20.86"/>
     <col customWidth="1" min="47" max="47" width="10.43"/>
     <col customWidth="1" min="48" max="48" width="23.0"/>
     <col customWidth="1" min="49" max="49" width="10.71"/>
@@ -4897,7 +4886,7 @@
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
       <c r="P2" s="3"/>
-      <c r="R2" s="34" t="s">
+      <c r="R2" s="28" t="s">
         <v>1</v>
       </c>
       <c r="S2" s="2"/>
@@ -4908,7 +4897,7 @@
       <c r="X2" s="2"/>
       <c r="Y2" s="2"/>
       <c r="Z2" s="3"/>
-      <c r="AB2" s="35" t="s">
+      <c r="AB2" s="29" t="s">
         <v>2</v>
       </c>
       <c r="AC2" s="2"/>
@@ -4919,8 +4908,8 @@
       <c r="AH2" s="2"/>
       <c r="AI2" s="2"/>
       <c r="AJ2" s="3"/>
-      <c r="AL2" s="36" t="s">
-        <v>174</v>
+      <c r="AL2" s="30" t="s">
+        <v>173</v>
       </c>
       <c r="AM2" s="2"/>
       <c r="AN2" s="2"/>
@@ -4928,7 +4917,7 @@
       <c r="AP2" s="2"/>
       <c r="AQ2" s="2"/>
       <c r="AR2" s="3"/>
-      <c r="AT2" s="37" t="s">
+      <c r="AT2" s="31" t="s">
         <v>4</v>
       </c>
       <c r="AU2" s="2"/>
@@ -4943,520 +4932,542 @@
       <c r="BD2" s="3"/>
     </row>
     <row r="4">
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="38" t="s">
-        <v>175</v>
-      </c>
-      <c r="F4" s="38" t="s">
+      <c r="D4" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="F4" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="38" t="s">
+      <c r="H4" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="38" t="s">
+      <c r="J4" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K4" s="12"/>
-      <c r="L4" s="38" t="s">
+      <c r="K4" s="11"/>
+      <c r="L4" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="M4" s="12"/>
-      <c r="N4" s="38" t="s">
+      <c r="M4" s="11"/>
+      <c r="N4" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="38" t="s">
+      <c r="O4" s="11"/>
+      <c r="P4" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="R4" s="39" t="s">
+      <c r="R4" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="T4" s="39" t="s">
+      <c r="T4" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="V4" s="39" t="s">
+      <c r="V4" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="X4" s="14" t="s">
+      <c r="X4" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="Z4" s="47" t="s">
+      <c r="Z4" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="AB4" s="41" t="s">
+      <c r="AB4" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="AD4" s="41" t="s">
+      <c r="AD4" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="AF4" s="41" t="s">
+      <c r="AF4" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="AH4" s="41" t="s">
+      <c r="AH4" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="AI4" s="12"/>
-      <c r="AJ4" s="48" t="s">
-        <v>221</v>
-      </c>
-      <c r="AL4" s="42" t="s">
+      <c r="AI4" s="11"/>
+      <c r="AJ4" s="35" t="s">
+        <v>214</v>
+      </c>
+      <c r="AL4" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="AN4" s="42" t="s">
+      <c r="AN4" s="36" t="s">
         <v>24</v>
       </c>
-      <c r="AP4" s="42" t="s">
+      <c r="AP4" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="AQ4" s="49"/>
-      <c r="AR4" s="42" t="s">
-        <v>222</v>
-      </c>
-      <c r="AT4" s="43" t="s">
+      <c r="AR4" s="43" t="s">
+        <v>215</v>
+      </c>
+      <c r="AT4" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="AU4" s="12"/>
-      <c r="AV4" s="43" t="s">
-        <v>223</v>
-      </c>
-      <c r="AX4" s="50" t="s">
+      <c r="AU4" s="11"/>
+      <c r="AV4" s="37" t="s">
+        <v>216</v>
+      </c>
+      <c r="AX4" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="AZ4" s="43" t="s">
+      <c r="AZ4" s="37" t="s">
         <v>28</v>
       </c>
-      <c r="BB4" s="43" t="s">
+      <c r="BB4" s="37" t="s">
         <v>29</v>
       </c>
-      <c r="BD4" s="43" t="s">
+      <c r="BD4" s="37" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="44" t="s">
+      <c r="B5" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="44" t="s">
-        <v>177</v>
-      </c>
-      <c r="F5" s="44" t="s">
+      <c r="D5" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="H5" s="22" t="s">
+      <c r="H5" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="44" t="s">
+      <c r="J5" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="K5" s="24"/>
-      <c r="L5" s="22" t="s">
+      <c r="K5" s="21"/>
+      <c r="L5" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="M5" s="24"/>
-      <c r="N5" s="22" t="s">
+      <c r="M5" s="21"/>
+      <c r="N5" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O5" s="24"/>
-      <c r="P5" s="22" t="s">
+      <c r="O5" s="21"/>
+      <c r="P5" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="R5" s="44" t="s">
-        <v>180</v>
-      </c>
-      <c r="T5" s="44" t="s">
+      <c r="R5" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="T5" s="19" t="s">
+        <v>217</v>
+      </c>
+      <c r="V5" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="V5" s="44" t="s">
-        <v>182</v>
-      </c>
-      <c r="X5" s="25" t="s">
+      <c r="X5" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="Z5" s="25" t="s">
+      <c r="Z5" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="AB5" s="44" t="s">
-        <v>183</v>
-      </c>
-      <c r="AD5" s="44" t="s">
-        <v>184</v>
-      </c>
-      <c r="AF5" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="AH5" s="22" t="s">
-        <v>225</v>
-      </c>
-      <c r="AI5" s="24"/>
-      <c r="AJ5" s="22" t="s">
-        <v>226</v>
-      </c>
-      <c r="AL5" s="25" t="s">
-        <v>188</v>
-      </c>
-      <c r="AN5" s="22" t="s">
+      <c r="AB5" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="AD5" s="19" t="s">
+        <v>185</v>
+      </c>
+      <c r="AF5" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="AH5" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="AI5" s="21"/>
+      <c r="AJ5" s="18" t="s">
+        <v>197</v>
+      </c>
+      <c r="AL5" s="22" t="s">
+        <v>187</v>
+      </c>
+      <c r="AN5" s="38" t="s">
+        <v>221</v>
+      </c>
+      <c r="AP5" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="AP5" s="22" t="s">
+      <c r="AR5" s="44" t="s">
+        <v>222</v>
+      </c>
+      <c r="AT5" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="AQ5" s="51"/>
-      <c r="AR5" s="22" t="s">
-        <v>227</v>
-      </c>
-      <c r="AT5" s="22" t="s">
-        <v>228</v>
-      </c>
-      <c r="AU5" s="24"/>
-      <c r="AV5" s="22" t="s">
-        <v>229</v>
-      </c>
-      <c r="AX5" s="22" t="s">
-        <v>230</v>
-      </c>
-      <c r="AZ5" s="44" t="s">
+      <c r="AU5" s="21"/>
+      <c r="AV5" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="AX5" s="18" t="s">
+        <v>191</v>
+      </c>
+      <c r="AZ5" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="BB5" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="BB5" s="44" t="s">
+      <c r="BD5" s="18" t="s">
         <v>194</v>
-      </c>
-      <c r="BD5" s="44" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="18" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="45" t="s">
+        <v>224</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>225</v>
+      </c>
+      <c r="H6" s="23" t="s">
+        <v>226</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="K6" s="21"/>
+      <c r="L6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="21"/>
+      <c r="N6" s="23" t="s">
+        <v>227</v>
+      </c>
+      <c r="O6" s="21"/>
+      <c r="P6" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="R6" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="T6" s="25" t="s">
+        <v>229</v>
+      </c>
+      <c r="V6" s="18" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="X6" s="24" t="s">
+        <v>230</v>
+      </c>
+      <c r="Z6" s="46" t="s">
         <v>231</v>
       </c>
-      <c r="F6" s="30" t="s">
+      <c r="AB6" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="AD6" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="AF6" s="23" t="s">
         <v>232</v>
       </c>
-      <c r="H6" s="27" t="s">
+      <c r="AH6" s="23" t="s">
+        <v>199</v>
+      </c>
+      <c r="AI6" s="21"/>
+      <c r="AJ6" s="38" t="s">
         <v>233</v>
       </c>
-      <c r="J6" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="K6" s="24"/>
-      <c r="L6" s="22" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" s="24"/>
-      <c r="N6" s="27" t="s">
+      <c r="AL6" s="22" t="s">
+        <v>186</v>
+      </c>
+      <c r="AN6" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="AP6" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="O6" s="24"/>
-      <c r="P6" s="27" t="s">
+      <c r="AR6" s="41" t="s">
         <v>235</v>
       </c>
-      <c r="R6" s="44" t="s">
-        <v>61</v>
-      </c>
-      <c r="T6" s="30" t="s">
+      <c r="AT6" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="AU6" s="21"/>
+      <c r="AV6" s="23" t="s">
         <v>236</v>
       </c>
-      <c r="V6" s="44" t="s">
-        <v>198</v>
-      </c>
-      <c r="X6" s="29" t="s">
+      <c r="AX6" s="25" t="s">
         <v>237</v>
       </c>
-      <c r="Z6" s="52" t="s">
+      <c r="AZ6" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="BB6" s="18" t="s">
+        <v>209</v>
+      </c>
+      <c r="BD6" s="38" t="s">
         <v>238</v>
-      </c>
-      <c r="AB6" s="44" t="s">
-        <v>199</v>
-      </c>
-      <c r="AD6" s="44" t="s">
-        <v>200</v>
-      </c>
-      <c r="AF6" s="27" t="s">
-        <v>239</v>
-      </c>
-      <c r="AH6" s="27" t="s">
-        <v>240</v>
-      </c>
-      <c r="AI6" s="24"/>
-      <c r="AJ6" s="22" t="s">
-        <v>241</v>
-      </c>
-      <c r="AL6" s="25" t="s">
-        <v>187</v>
-      </c>
-      <c r="AN6" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="AP6" s="45" t="s">
-        <v>204</v>
-      </c>
-      <c r="AQ6" s="53"/>
-      <c r="AR6" s="54" t="s">
-        <v>242</v>
-      </c>
-      <c r="AT6" s="22" t="s">
-        <v>243</v>
-      </c>
-      <c r="AU6" s="24"/>
-      <c r="AV6" s="27" t="s">
-        <v>244</v>
-      </c>
-      <c r="AX6" s="30" t="s">
-        <v>245</v>
-      </c>
-      <c r="AZ6" s="26" t="s">
-        <v>80</v>
-      </c>
-      <c r="BB6" s="22" t="s">
-        <v>246</v>
-      </c>
-      <c r="BD6" s="27" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="D7" s="55"/>
-      <c r="F7" s="31"/>
-      <c r="H7" s="12"/>
-      <c r="J7" s="26" t="s">
+      <c r="D7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="H7" s="11"/>
+      <c r="J7" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="K7" s="12"/>
-      <c r="L7" s="22" t="s">
+      <c r="K7" s="11"/>
+      <c r="L7" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="M7" s="12"/>
-      <c r="N7" s="32"/>
-      <c r="O7" s="12"/>
-      <c r="P7" s="12"/>
-      <c r="R7" s="44" t="s">
-        <v>208</v>
-      </c>
-      <c r="T7" s="55"/>
-      <c r="V7" s="44" t="s">
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="11"/>
+      <c r="P7" s="11"/>
+      <c r="R7" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="T7" s="26"/>
+      <c r="V7" s="18" t="s">
         <v>77</v>
       </c>
-      <c r="X7" s="22" t="s">
-        <v>138</v>
-      </c>
-      <c r="Z7" s="56"/>
-      <c r="AB7" s="26" t="s">
-        <v>209</v>
-      </c>
-      <c r="AD7" s="27" t="s">
-        <v>248</v>
-      </c>
-      <c r="AF7" s="25" t="s">
-        <v>249</v>
-      </c>
-      <c r="AH7" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="AI7" s="12"/>
-      <c r="AJ7" s="12"/>
-      <c r="AL7" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="AN7" s="26" t="s">
-        <v>102</v>
-      </c>
-      <c r="AP7" s="45" t="s">
-        <v>250</v>
-      </c>
-      <c r="AQ7" s="53"/>
-      <c r="AR7" s="57"/>
-      <c r="AT7" s="44" t="s">
+      <c r="X7" s="18" t="s">
+        <v>137</v>
+      </c>
+      <c r="Z7" s="47"/>
+      <c r="AB7" s="23" t="s">
+        <v>240</v>
+      </c>
+      <c r="AD7" s="19" t="s">
+        <v>241</v>
+      </c>
+      <c r="AF7" s="22" t="s">
+        <v>242</v>
+      </c>
+      <c r="AH7" s="23" t="s">
+        <v>122</v>
+      </c>
+      <c r="AI7" s="11"/>
+      <c r="AJ7" s="11"/>
+      <c r="AL7" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="AN7" s="19" t="s">
+        <v>243</v>
+      </c>
+      <c r="AP7" s="48" t="s">
+        <v>244</v>
+      </c>
+      <c r="AT7" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="AU7" s="24"/>
-      <c r="AV7" s="49"/>
-      <c r="AX7" s="55"/>
-      <c r="AZ7" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="BB7" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="BD7" s="12"/>
+      <c r="AU7" s="21"/>
+      <c r="AV7" s="48" t="s">
+        <v>245</v>
+      </c>
+      <c r="AX7" s="26"/>
+      <c r="BB7" s="23" t="s">
+        <v>154</v>
+      </c>
+      <c r="BD7" s="11"/>
     </row>
     <row r="8">
-      <c r="B8" s="44" t="s">
-        <v>109</v>
-      </c>
-      <c r="D8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="J8" s="26" t="s">
-        <v>133</v>
-      </c>
-      <c r="K8" s="12"/>
-      <c r="L8" s="22" t="s">
-        <v>114</v>
-      </c>
-      <c r="M8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="32"/>
-      <c r="R8" s="26" t="s">
-        <v>116</v>
-      </c>
-      <c r="T8" s="12"/>
-      <c r="V8" s="26" t="s">
-        <v>118</v>
+      <c r="B8" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="D8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="J8" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="K8" s="11"/>
+      <c r="L8" s="18" t="s">
+        <v>113</v>
+      </c>
+      <c r="M8" s="11"/>
+      <c r="O8" s="11"/>
+      <c r="P8" s="11"/>
+      <c r="R8" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="T8" s="11"/>
+      <c r="V8" s="23" t="s">
+        <v>117</v>
       </c>
       <c r="Z8" s="49"/>
-      <c r="AB8" s="26" t="s">
-        <v>212</v>
-      </c>
-      <c r="AD8" s="26" t="s">
-        <v>210</v>
-      </c>
-      <c r="AH8" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="AI8" s="12"/>
-      <c r="AJ8" s="12"/>
-      <c r="AL8" s="29" t="s">
+      <c r="AB8" s="23" t="s">
+        <v>246</v>
+      </c>
+      <c r="AD8" s="23" t="s">
+        <v>208</v>
+      </c>
+      <c r="AH8" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="AI8" s="11"/>
+      <c r="AJ8" s="11"/>
+      <c r="AL8" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="AN8" s="23" t="s">
         <v>125</v>
       </c>
-      <c r="AN8" s="26" t="s">
-        <v>126</v>
-      </c>
-      <c r="AR8" s="57"/>
-      <c r="AT8" s="27" t="s">
-        <v>128</v>
-      </c>
-      <c r="AU8" s="12"/>
-      <c r="AV8" s="32"/>
-      <c r="BB8" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="BD8" s="12"/>
+      <c r="AP8" s="50" t="s">
+        <v>186</v>
+      </c>
+      <c r="AT8" s="23" t="s">
+        <v>127</v>
+      </c>
+      <c r="AU8" s="11"/>
+      <c r="AV8" s="11"/>
+      <c r="BB8" s="23" t="s">
+        <v>160</v>
+      </c>
+      <c r="BD8" s="11"/>
     </row>
     <row r="9">
-      <c r="B9" s="44" t="s">
-        <v>252</v>
-      </c>
-      <c r="D9" s="32"/>
-      <c r="J9" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="26" t="s">
+      <c r="B9" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="D9" s="11"/>
+      <c r="J9" s="23" t="s">
+        <v>147</v>
+      </c>
+      <c r="K9" s="11"/>
+      <c r="L9" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="M9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="R9" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="M9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="R9" s="26" t="s">
-        <v>135</v>
-      </c>
-      <c r="T9" s="12"/>
-      <c r="V9" s="26" t="s">
-        <v>137</v>
-      </c>
-      <c r="AL9" s="29" t="s">
-        <v>142</v>
-      </c>
-      <c r="AR9" s="57"/>
-      <c r="AT9" s="27" t="s">
-        <v>144</v>
-      </c>
-      <c r="AU9" s="12"/>
-      <c r="AV9" s="32"/>
-      <c r="BB9" s="26" t="s">
-        <v>167</v>
-      </c>
-      <c r="BD9" s="12"/>
+      <c r="T9" s="11"/>
+      <c r="V9" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB9" s="23" t="s">
+        <v>138</v>
+      </c>
+      <c r="AL9" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="AN9" s="19" t="s">
+        <v>249</v>
+      </c>
+      <c r="AP9" s="51" t="s">
+        <v>250</v>
+      </c>
+      <c r="AT9" s="23" t="s">
+        <v>143</v>
+      </c>
+      <c r="AU9" s="11"/>
+      <c r="AV9" s="11"/>
+      <c r="BB9" s="23" t="s">
+        <v>166</v>
+      </c>
+      <c r="BD9" s="11"/>
     </row>
     <row r="10">
-      <c r="B10" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="D10" s="32"/>
-      <c r="J10" s="27" t="s">
-        <v>113</v>
-      </c>
-      <c r="L10" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="R10" s="25" t="s">
-        <v>253</v>
-      </c>
-      <c r="AR10" s="32"/>
-      <c r="AT10" s="27" t="s">
-        <v>154</v>
-      </c>
-      <c r="AU10" s="12"/>
-      <c r="AV10" s="32"/>
-      <c r="BB10" s="22" t="s">
-        <v>254</v>
+      <c r="B10" s="19" t="s">
+        <v>234</v>
+      </c>
+      <c r="D10" s="11"/>
+      <c r="J10" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="L10" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="R10" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="AB10" s="23" t="s">
+        <v>150</v>
+      </c>
+      <c r="AL10" s="24" t="s">
+        <v>141</v>
+      </c>
+      <c r="AT10" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="AU10" s="11"/>
+      <c r="AV10" s="11"/>
+      <c r="BB10" s="18" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="26" t="s">
-        <v>215</v>
-      </c>
-      <c r="D11" s="32"/>
-      <c r="L11" s="27" t="s">
-        <v>157</v>
-      </c>
-      <c r="T11" s="12"/>
-      <c r="AT11" s="27" t="s">
-        <v>160</v>
-      </c>
-      <c r="AU11" s="12"/>
-      <c r="AV11" s="12"/>
-      <c r="BB11" s="29" t="s">
-        <v>169</v>
+      <c r="B11" s="23" t="s">
+        <v>146</v>
+      </c>
+      <c r="D11" s="11"/>
+      <c r="L11" s="23" t="s">
+        <v>156</v>
+      </c>
+      <c r="T11" s="11"/>
+      <c r="AT11" s="23" t="s">
+        <v>159</v>
+      </c>
+      <c r="AU11" s="11"/>
+      <c r="AV11" s="11"/>
+      <c r="BB11" s="24" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="26" t="s">
-        <v>165</v>
-      </c>
-      <c r="AT12" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="AU12" s="12"/>
-      <c r="AV12" s="12"/>
+      <c r="B12" s="23" t="s">
+        <v>212</v>
+      </c>
+      <c r="AT12" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="AU12" s="11"/>
+      <c r="AV12" s="11"/>
+      <c r="BB12" s="50" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="13">
-      <c r="B13" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="AT13" s="44" t="s">
-        <v>214</v>
-      </c>
-      <c r="AU13" s="12"/>
-      <c r="AV13" s="12"/>
+      <c r="B13" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="AT13" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="AU13" s="11"/>
+      <c r="BB13" s="50" t="s">
+        <v>254</v>
+      </c>
     </row>
     <row r="14">
-      <c r="B14" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="AT14" s="44" t="s">
-        <v>211</v>
+      <c r="B14" s="23" t="s">
+        <v>167</v>
+      </c>
+      <c r="AT14" s="18" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="26" t="s">
-        <v>171</v>
+      <c r="B15" s="23" t="s">
+        <v>169</v>
+      </c>
+      <c r="AT15" s="19" t="s">
+        <v>255</v>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="29" t="s">
-        <v>173</v>
+      <c r="B16" s="23" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="24" t="s">
         <v>172</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="23" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -6441,11 +6452,11 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="5">
+    <mergeCell ref="B2:P2"/>
     <mergeCell ref="R2:Z2"/>
     <mergeCell ref="AB2:AJ2"/>
     <mergeCell ref="AL2:AR2"/>
     <mergeCell ref="AT2:BD2"/>
-    <mergeCell ref="B2:P2"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>